<commit_message>
Arrays in  JAVA commit
</commit_message>
<xml_diff>
--- a/DailyTrack.xlsx
+++ b/DailyTrack.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="39">
   <si>
     <t>https://leetcode.com/problems/transpose-matrix/submissions/1904630410/</t>
   </si>
@@ -70,13 +70,76 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/maximum-of-all-subarrays-of-size-k3101/0</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/rotate-image/description/</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/rotate-by-90-degree0356/1</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/rotate-by-90-degree-1587115621/1</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/pascals-triangle/description/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/pascals-triangle-ii/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/search-a-2d-matrix-ii/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/trionic-array-i/submissions/1906295827/?envType=daily-question&amp;envId=2026-02-03</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/spirally-traversing-a-matrix-1587115621/1</t>
+  </si>
+  <si>
+    <t>FarmXChain</t>
+  </si>
+  <si>
+    <t>Portfolio</t>
+  </si>
+  <si>
+    <t>Focus_Clock</t>
+  </si>
+  <si>
+    <t>Fashion Sense</t>
+  </si>
+  <si>
+    <t>Fake News</t>
+  </si>
+  <si>
+    <t>Spliter-AI</t>
+  </si>
+  <si>
+    <t>https://personalized-clock.vercel.app/</t>
+  </si>
+  <si>
+    <t>https://final-year-project-1-lyart.vercel.app/</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Have to Start</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/check-if-an-array-is-sorted0701/1</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/move-all-zeroes-to-end-of-array0751/1</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-removals-to-balance-array/submissions/1909919948/?envType=daily-question&amp;envId=2026-02-06</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -87,6 +150,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -139,18 +210,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -450,10 +525,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:I11"/>
+  <dimension ref="B1:I22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="71.6640625" customWidth="1"/>
+    <col min="4" max="4" width="100" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:9" x14ac:dyDescent="0.3">
@@ -463,7 +538,7 @@
       <c r="C1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="6" t="s">
         <v>10</v>
       </c>
     </row>
@@ -471,7 +546,7 @@
       <c r="C2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="6" t="s">
         <v>13</v>
       </c>
     </row>
@@ -479,7 +554,7 @@
       <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="6" t="s">
         <v>11</v>
       </c>
       <c r="H3" s="4"/>
@@ -491,7 +566,7 @@
       <c r="C4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="6" t="s">
         <v>12</v>
       </c>
       <c r="H4" s="1"/>
@@ -503,7 +578,7 @@
       <c r="C5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="6" t="s">
         <v>14</v>
       </c>
       <c r="H5" s="5"/>
@@ -515,7 +590,7 @@
       <c r="C6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="6" t="s">
         <v>15</v>
       </c>
       <c r="H6" s="2"/>
@@ -527,7 +602,7 @@
       <c r="C7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="6" t="s">
         <v>16</v>
       </c>
     </row>
@@ -535,7 +610,7 @@
       <c r="C8" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="6" t="s">
         <v>17</v>
       </c>
     </row>
@@ -546,7 +621,7 @@
       <c r="C10" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="6" t="s">
         <v>0</v>
       </c>
     </row>
@@ -554,21 +629,185 @@
       <c r="C11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="6" t="s">
         <v>4</v>
       </c>
     </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C13" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C14" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C17" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C19" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C20" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C21" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="22" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C22" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D17" r:id="rId1"/>
+    <hyperlink ref="D16" r:id="rId2"/>
+    <hyperlink ref="D15" r:id="rId3"/>
+    <hyperlink ref="D14" r:id="rId4"/>
+    <hyperlink ref="D13" r:id="rId5"/>
+    <hyperlink ref="D12" r:id="rId6"/>
+    <hyperlink ref="D11" r:id="rId7"/>
+    <hyperlink ref="D10" r:id="rId8"/>
+    <hyperlink ref="D8" r:id="rId9"/>
+    <hyperlink ref="D7" r:id="rId10"/>
+    <hyperlink ref="D6" r:id="rId11"/>
+    <hyperlink ref="D5" r:id="rId12"/>
+    <hyperlink ref="D4" r:id="rId13"/>
+    <hyperlink ref="D3" r:id="rId14"/>
+    <hyperlink ref="D2" r:id="rId15"/>
+    <hyperlink ref="D1" r:id="rId16"/>
+    <hyperlink ref="D18" r:id="rId17"/>
+    <hyperlink ref="D19" r:id="rId18"/>
+    <hyperlink ref="D20" r:id="rId19"/>
+    <hyperlink ref="D21" r:id="rId20"/>
+    <hyperlink ref="D22" r:id="rId21"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId22"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A2:B7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="17.77734375" customWidth="1"/>
+    <col min="2" max="2" width="71.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>